<commit_message>
Include per-step tick/cross summary in notification email
</commit_message>
<xml_diff>
--- a/Wheelo_Team_Data.xlsx
+++ b/Wheelo_Team_Data.xlsx
@@ -2020,7 +2020,7 @@
         <v>1532.2</v>
       </c>
       <c r="J2" t="n">
-        <v>9.75</v>
+        <v>12.4</v>
       </c>
       <c r="K2" t="n">
         <v>46.594</v>
@@ -2392,7 +2392,7 @@
         <v>1547.6</v>
       </c>
       <c r="ED2" t="n">
-        <v>20.25</v>
+        <v>17.6</v>
       </c>
       <c r="EE2" t="n">
         <v>40</v>
@@ -2722,7 +2722,7 @@
         <v>-15.4</v>
       </c>
       <c r="IJ2" t="n">
-        <v>-10.5</v>
+        <v>-5.2</v>
       </c>
       <c r="IK2" t="n">
         <v>0.2</v>
@@ -3894,7 +3894,7 @@
         <v>1620</v>
       </c>
       <c r="J4" t="n">
-        <v>16.75</v>
+        <v>17.2</v>
       </c>
       <c r="K4" t="n">
         <v>52.427</v>
@@ -4266,7 +4266,7 @@
         <v>1451.2</v>
       </c>
       <c r="ED4" t="n">
-        <v>13.25</v>
+        <v>12.8</v>
       </c>
       <c r="EE4" t="n">
         <v>39.2</v>
@@ -4596,7 +4596,7 @@
         <v>168.8</v>
       </c>
       <c r="IJ4" t="n">
-        <v>3.5</v>
+        <v>4.4</v>
       </c>
       <c r="IK4" t="n">
         <v>5</v>
@@ -4833,7 +4833,7 @@
         <v>1472.8</v>
       </c>
       <c r="J5" t="n">
-        <v>8</v>
+        <v>7.8</v>
       </c>
       <c r="K5" t="n">
         <v>46.252</v>
@@ -5205,7 +5205,7 @@
         <v>1568.4</v>
       </c>
       <c r="ED5" t="n">
-        <v>22</v>
+        <v>22.2</v>
       </c>
       <c r="EE5" t="n">
         <v>41.6</v>
@@ -5535,7 +5535,7 @@
         <v>-95.59999999999999</v>
       </c>
       <c r="IJ5" t="n">
-        <v>-14</v>
+        <v>-14.4</v>
       </c>
       <c r="IK5" t="n">
         <v>-1.6</v>
@@ -5772,7 +5772,7 @@
         <v>1551.2</v>
       </c>
       <c r="J6" t="n">
-        <v>13.25</v>
+        <v>12.6</v>
       </c>
       <c r="K6" t="n">
         <v>48.664</v>
@@ -6144,7 +6144,7 @@
         <v>1637.8</v>
       </c>
       <c r="ED6" t="n">
-        <v>16.75</v>
+        <v>17.4</v>
       </c>
       <c r="EE6" t="n">
         <v>45</v>
@@ -6474,7 +6474,7 @@
         <v>-86.59999999999999</v>
       </c>
       <c r="IJ6" t="n">
-        <v>-3.5</v>
+        <v>-4.8</v>
       </c>
       <c r="IK6" t="n">
         <v>-5.4</v>
@@ -6711,7 +6711,7 @@
         <v>1451.2</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>7.4</v>
       </c>
       <c r="K7" t="n">
         <v>45.487</v>
@@ -7083,7 +7083,7 @@
         <v>1693.2</v>
       </c>
       <c r="ED7" t="n">
-        <v>28</v>
+        <v>22.6</v>
       </c>
       <c r="EE7" t="n">
         <v>45.6</v>
@@ -7413,7 +7413,7 @@
         <v>-242</v>
       </c>
       <c r="IJ7" t="n">
-        <v>-26</v>
+        <v>-15.2</v>
       </c>
       <c r="IK7" t="n">
         <v>-5.4</v>
@@ -7650,7 +7650,7 @@
         <v>1527</v>
       </c>
       <c r="J8" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="K8" t="n">
         <v>49.709</v>
@@ -8022,7 +8022,7 @@
         <v>1478.6</v>
       </c>
       <c r="ED8" t="n">
-        <v>8.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="EE8" t="n">
         <v>39.6</v>
@@ -8352,7 +8352,7 @@
         <v>48.4</v>
       </c>
       <c r="IJ8" t="n">
-        <v>13</v>
+        <v>12.4</v>
       </c>
       <c r="IK8" t="n">
         <v>3.6</v>
@@ -8589,7 +8589,7 @@
         <v>1621.4</v>
       </c>
       <c r="J9" t="n">
-        <v>13</v>
+        <v>16.4</v>
       </c>
       <c r="K9" t="n">
         <v>52.559</v>
@@ -8961,7 +8961,7 @@
         <v>1470.6</v>
       </c>
       <c r="ED9" t="n">
-        <v>17</v>
+        <v>13.6</v>
       </c>
       <c r="EE9" t="n">
         <v>40.2</v>
@@ -9291,7 +9291,7 @@
         <v>150.8</v>
       </c>
       <c r="IJ9" t="n">
-        <v>-4</v>
+        <v>2.8</v>
       </c>
       <c r="IK9" t="n">
         <v>2.2</v>
@@ -9528,7 +9528,7 @@
         <v>1508.8</v>
       </c>
       <c r="J10" t="n">
-        <v>22.25</v>
+        <v>17.8</v>
       </c>
       <c r="K10" t="n">
         <v>53.818</v>
@@ -9900,7 +9900,7 @@
         <v>1520.2</v>
       </c>
       <c r="ED10" t="n">
-        <v>7.75</v>
+        <v>12.2</v>
       </c>
       <c r="EE10" t="n">
         <v>40.4</v>
@@ -10230,7 +10230,7 @@
         <v>-11.4</v>
       </c>
       <c r="IJ10" t="n">
-        <v>14.5</v>
+        <v>5.6</v>
       </c>
       <c r="IK10" t="n">
         <v>1.8</v>
@@ -10467,7 +10467,7 @@
         <v>1618.2</v>
       </c>
       <c r="J11" t="n">
-        <v>11.5</v>
+        <v>15.2</v>
       </c>
       <c r="K11" t="n">
         <v>50.94</v>
@@ -10839,7 +10839,7 @@
         <v>1490.6</v>
       </c>
       <c r="ED11" t="n">
-        <v>18.5</v>
+        <v>14.8</v>
       </c>
       <c r="EE11" t="n">
         <v>40.6</v>
@@ -11169,7 +11169,7 @@
         <v>127.6</v>
       </c>
       <c r="IJ11" t="n">
-        <v>-7</v>
+        <v>0.4</v>
       </c>
       <c r="IK11" t="n">
         <v>2.6</v>
@@ -11406,7 +11406,7 @@
         <v>1696.6</v>
       </c>
       <c r="J12" t="n">
-        <v>20.25</v>
+        <v>22</v>
       </c>
       <c r="K12" t="n">
         <v>53.937</v>
@@ -11778,7 +11778,7 @@
         <v>1430</v>
       </c>
       <c r="ED12" t="n">
-        <v>9.75</v>
+        <v>8</v>
       </c>
       <c r="EE12" t="n">
         <v>37.6</v>
@@ -12108,7 +12108,7 @@
         <v>266.6</v>
       </c>
       <c r="IJ12" t="n">
-        <v>10.5</v>
+        <v>14</v>
       </c>
       <c r="IK12" t="n">
         <v>8.6</v>
@@ -12345,7 +12345,7 @@
         <v>1505.8</v>
       </c>
       <c r="J13" t="n">
-        <v>20.75</v>
+        <v>16.8</v>
       </c>
       <c r="K13" t="n">
         <v>52.381</v>
@@ -12717,7 +12717,7 @@
         <v>1616.8</v>
       </c>
       <c r="ED13" t="n">
-        <v>9.25</v>
+        <v>13.2</v>
       </c>
       <c r="EE13" t="n">
         <v>44.4</v>
@@ -13047,7 +13047,7 @@
         <v>-111</v>
       </c>
       <c r="IJ13" t="n">
-        <v>11.5</v>
+        <v>3.6</v>
       </c>
       <c r="IK13" t="n">
         <v>-5.2</v>
@@ -13284,7 +13284,7 @@
         <v>1559.2</v>
       </c>
       <c r="J14" t="n">
-        <v>23</v>
+        <v>20.6</v>
       </c>
       <c r="K14" t="n">
         <v>47.352</v>
@@ -13656,7 +13656,7 @@
         <v>1409</v>
       </c>
       <c r="ED14" t="n">
-        <v>7</v>
+        <v>9.4</v>
       </c>
       <c r="EE14" t="n">
         <v>40.2</v>
@@ -13986,7 +13986,7 @@
         <v>150.2</v>
       </c>
       <c r="IJ14" t="n">
-        <v>16</v>
+        <v>11.2</v>
       </c>
       <c r="IK14" t="n">
         <v>3.6</v>
@@ -14223,7 +14223,7 @@
         <v>1532</v>
       </c>
       <c r="J15" t="n">
-        <v>16.75</v>
+        <v>16</v>
       </c>
       <c r="K15" t="n">
         <v>53.747</v>
@@ -14595,7 +14595,7 @@
         <v>1445.4</v>
       </c>
       <c r="ED15" t="n">
-        <v>13.25</v>
+        <v>14</v>
       </c>
       <c r="EE15" t="n">
         <v>41.6</v>
@@ -14925,7 +14925,7 @@
         <v>86.59999999999999</v>
       </c>
       <c r="IJ15" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="IK15" t="n">
         <v>2.2</v>
@@ -15162,7 +15162,7 @@
         <v>1359.2</v>
       </c>
       <c r="J16" t="n">
-        <v>2.25</v>
+        <v>1.8</v>
       </c>
       <c r="K16" t="n">
         <v>47.037</v>
@@ -15534,7 +15534,7 @@
         <v>1588.6</v>
       </c>
       <c r="ED16" t="n">
-        <v>27.75</v>
+        <v>28.2</v>
       </c>
       <c r="EE16" t="n">
         <v>45.6</v>
@@ -15864,7 +15864,7 @@
         <v>-229.4</v>
       </c>
       <c r="IJ16" t="n">
-        <v>-25.5</v>
+        <v>-26.4</v>
       </c>
       <c r="IK16" t="n">
         <v>-7.8</v>
@@ -16101,7 +16101,7 @@
         <v>1554.6</v>
       </c>
       <c r="J17" t="n">
-        <v>11.75</v>
+        <v>12.8</v>
       </c>
       <c r="K17" t="n">
         <v>48.829</v>
@@ -16473,7 +16473,7 @@
         <v>1628.8</v>
       </c>
       <c r="ED17" t="n">
-        <v>18.25</v>
+        <v>17.2</v>
       </c>
       <c r="EE17" t="n">
         <v>43</v>
@@ -16803,7 +16803,7 @@
         <v>-74.2</v>
       </c>
       <c r="IJ17" t="n">
-        <v>-6.5</v>
+        <v>-4.4</v>
       </c>
       <c r="IK17" t="n">
         <v>-1.8</v>
@@ -17040,7 +17040,7 @@
         <v>1598.8</v>
       </c>
       <c r="J18" t="n">
-        <v>21.75</v>
+        <v>23.4</v>
       </c>
       <c r="K18" t="n">
         <v>54.101</v>
@@ -17412,7 +17412,7 @@
         <v>1381.6</v>
       </c>
       <c r="ED18" t="n">
-        <v>8.25</v>
+        <v>6.6</v>
       </c>
       <c r="EE18" t="n">
         <v>40.8</v>
@@ -17742,7 +17742,7 @@
         <v>217.2</v>
       </c>
       <c r="IJ18" t="n">
-        <v>13.5</v>
+        <v>16.8</v>
       </c>
       <c r="IK18" t="n">
         <v>2.4</v>
@@ -17979,7 +17979,7 @@
         <v>1347.8</v>
       </c>
       <c r="J19" t="n">
-        <v>10.5</v>
+        <v>8.4</v>
       </c>
       <c r="K19" t="n">
         <v>45.364</v>
@@ -18351,7 +18351,7 @@
         <v>1599.6</v>
       </c>
       <c r="ED19" t="n">
-        <v>19.5</v>
+        <v>21.6</v>
       </c>
       <c r="EE19" t="n">
         <v>43.6</v>
@@ -18681,7 +18681,7 @@
         <v>-251.8</v>
       </c>
       <c r="IJ19" t="n">
-        <v>-9</v>
+        <v>-13.2</v>
       </c>
       <c r="IK19" t="n">
         <v>-3</v>
@@ -18918,7 +18918,7 @@
         <v>1548.2</v>
       </c>
       <c r="J20" t="n">
-        <v>25</v>
+        <v>20.2</v>
       </c>
       <c r="K20" t="n">
         <v>50.801</v>
@@ -19290,7 +19290,7 @@
         <v>1647</v>
       </c>
       <c r="ED20" t="n">
-        <v>5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="EE20" t="n">
         <v>42.8</v>
@@ -19620,7 +19620,7 @@
         <v>-98.8</v>
       </c>
       <c r="IJ20" t="n">
-        <v>20</v>
+        <v>10.4</v>
       </c>
       <c r="IK20" t="n">
         <v>-2</v>
@@ -21428,7 +21428,7 @@
         <v>1486.9</v>
       </c>
       <c r="J2" t="n">
-        <v>9.778</v>
+        <v>11.1</v>
       </c>
       <c r="K2" t="n">
         <v>46.879</v>
@@ -21800,7 +21800,7 @@
         <v>1527.7</v>
       </c>
       <c r="ED2" t="n">
-        <v>20.222</v>
+        <v>18.9</v>
       </c>
       <c r="EE2" t="n">
         <v>41.7</v>
@@ -22130,7 +22130,7 @@
         <v>-40.8</v>
       </c>
       <c r="IJ2" t="n">
-        <v>-10.444</v>
+        <v>-7.8</v>
       </c>
       <c r="IK2" t="n">
         <v>-2.5</v>
@@ -22367,7 +22367,7 @@
         <v>1507.061</v>
       </c>
       <c r="J3" t="n">
-        <v>14.241</v>
+        <v>14.317</v>
       </c>
       <c r="K3" t="n">
         <v>49.662</v>
@@ -22735,7 +22735,7 @@
         <v>1525.539</v>
       </c>
       <c r="ED3" t="n">
-        <v>15.944</v>
+        <v>15.85</v>
       </c>
       <c r="EE3" t="n">
         <v>41.611</v>
@@ -23065,7 +23065,7 @@
         <v>-18.478</v>
       </c>
       <c r="IJ3" t="n">
-        <v>-1.704</v>
+        <v>-1.533</v>
       </c>
       <c r="IK3" t="n">
         <v>-0.417</v>
@@ -23302,7 +23302,7 @@
         <v>1647.8</v>
       </c>
       <c r="J4" t="n">
-        <v>22</v>
+        <v>21.7</v>
       </c>
       <c r="K4" t="n">
         <v>51.333</v>
@@ -23674,7 +23674,7 @@
         <v>1432.2</v>
       </c>
       <c r="ED4" t="n">
-        <v>9.667</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="EE4" t="n">
         <v>39.2</v>
@@ -24004,7 +24004,7 @@
         <v>215.6</v>
       </c>
       <c r="IJ4" t="n">
-        <v>12.333</v>
+        <v>11.9</v>
       </c>
       <c r="IK4" t="n">
         <v>3.3</v>
@@ -24241,7 +24241,7 @@
         <v>1485.6</v>
       </c>
       <c r="J5" t="n">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="K5" t="n">
         <v>49.305</v>
@@ -24613,7 +24613,7 @@
         <v>1523.3</v>
       </c>
       <c r="ED5" t="n">
-        <v>18</v>
+        <v>18.5</v>
       </c>
       <c r="EE5" t="n">
         <v>42.1</v>
@@ -24943,7 +24943,7 @@
         <v>-37.7</v>
       </c>
       <c r="IJ5" t="n">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="IK5" t="n">
         <v>-1.9</v>
@@ -25180,7 +25180,7 @@
         <v>1501.9</v>
       </c>
       <c r="J6" t="n">
-        <v>13.111</v>
+        <v>12.8</v>
       </c>
       <c r="K6" t="n">
         <v>50.471</v>
@@ -25552,7 +25552,7 @@
         <v>1596.1</v>
       </c>
       <c r="ED6" t="n">
-        <v>16.889</v>
+        <v>17.2</v>
       </c>
       <c r="EE6" t="n">
         <v>43.1</v>
@@ -25882,7 +25882,7 @@
         <v>-94.2</v>
       </c>
       <c r="IJ6" t="n">
-        <v>-3.778</v>
+        <v>-4.4</v>
       </c>
       <c r="IK6" t="n">
         <v>-2.3</v>
@@ -26119,7 +26119,7 @@
         <v>1432.9</v>
       </c>
       <c r="J7" t="n">
-        <v>4.444</v>
+        <v>6.9</v>
       </c>
       <c r="K7" t="n">
         <v>44.883</v>
@@ -26491,7 +26491,7 @@
         <v>1635.1</v>
       </c>
       <c r="ED7" t="n">
-        <v>25.556</v>
+        <v>23.1</v>
       </c>
       <c r="EE7" t="n">
         <v>45.2</v>
@@ -26821,7 +26821,7 @@
         <v>-202.2</v>
       </c>
       <c r="IJ7" t="n">
-        <v>-21.111</v>
+        <v>-16.2</v>
       </c>
       <c r="IK7" t="n">
         <v>-5.7</v>
@@ -27058,7 +27058,7 @@
         <v>1439.3</v>
       </c>
       <c r="J8" t="n">
-        <v>16.556</v>
+        <v>16.9</v>
       </c>
       <c r="K8" t="n">
         <v>49.522</v>
@@ -27430,7 +27430,7 @@
         <v>1518.6</v>
       </c>
       <c r="ED8" t="n">
-        <v>13.444</v>
+        <v>13.1</v>
       </c>
       <c r="EE8" t="n">
         <v>41.1</v>
@@ -27760,7 +27760,7 @@
         <v>-79.3</v>
       </c>
       <c r="IJ8" t="n">
-        <v>3.111</v>
+        <v>3.8</v>
       </c>
       <c r="IK8" t="n">
         <v>0.5</v>
@@ -27997,7 +27997,7 @@
         <v>1581.2</v>
       </c>
       <c r="J9" t="n">
-        <v>18.667</v>
+        <v>19.8</v>
       </c>
       <c r="K9" t="n">
         <v>52.821</v>
@@ -28369,7 +28369,7 @@
         <v>1507</v>
       </c>
       <c r="ED9" t="n">
-        <v>13</v>
+        <v>11.7</v>
       </c>
       <c r="EE9" t="n">
         <v>39.5</v>
@@ -28699,7 +28699,7 @@
         <v>74.2</v>
       </c>
       <c r="IJ9" t="n">
-        <v>5.667</v>
+        <v>8.1</v>
       </c>
       <c r="IK9" t="n">
         <v>2.1</v>
@@ -28936,7 +28936,7 @@
         <v>1451</v>
       </c>
       <c r="J10" t="n">
-        <v>16.111</v>
+        <v>14.5</v>
       </c>
       <c r="K10" t="n">
         <v>53.045</v>
@@ -29308,7 +29308,7 @@
         <v>1504.2</v>
       </c>
       <c r="ED10" t="n">
-        <v>13.889</v>
+        <v>15.5</v>
       </c>
       <c r="EE10" t="n">
         <v>41.1</v>
@@ -29638,7 +29638,7 @@
         <v>-53.2</v>
       </c>
       <c r="IJ10" t="n">
-        <v>2.222</v>
+        <v>-1</v>
       </c>
       <c r="IK10" t="n">
         <v>0.4</v>
@@ -29875,7 +29875,7 @@
         <v>1561.7</v>
       </c>
       <c r="J11" t="n">
-        <v>14.889</v>
+        <v>16.4</v>
       </c>
       <c r="K11" t="n">
         <v>49.585</v>
@@ -30247,7 +30247,7 @@
         <v>1454.8</v>
       </c>
       <c r="ED11" t="n">
-        <v>15.111</v>
+        <v>13.6</v>
       </c>
       <c r="EE11" t="n">
         <v>40.9</v>
@@ -30577,7 +30577,7 @@
         <v>106.9</v>
       </c>
       <c r="IJ11" t="n">
-        <v>-0.222</v>
+        <v>2.8</v>
       </c>
       <c r="IK11" t="n">
         <v>0.9</v>
@@ -30814,7 +30814,7 @@
         <v>1601.2</v>
       </c>
       <c r="J12" t="n">
-        <v>17.111</v>
+        <v>18.3</v>
       </c>
       <c r="K12" t="n">
         <v>51.939</v>
@@ -31186,7 +31186,7 @@
         <v>1487.9</v>
       </c>
       <c r="ED12" t="n">
-        <v>12.889</v>
+        <v>11.7</v>
       </c>
       <c r="EE12" t="n">
         <v>38.3</v>
@@ -31516,7 +31516,7 @@
         <v>113.3</v>
       </c>
       <c r="IJ12" t="n">
-        <v>4.222</v>
+        <v>6.6</v>
       </c>
       <c r="IK12" t="n">
         <v>5.3</v>
@@ -31753,7 +31753,7 @@
         <v>1539.9</v>
       </c>
       <c r="J13" t="n">
-        <v>17</v>
+        <v>15.4</v>
       </c>
       <c r="K13" t="n">
         <v>52.027</v>
@@ -32125,7 +32125,7 @@
         <v>1572.8</v>
       </c>
       <c r="ED13" t="n">
-        <v>13</v>
+        <v>14.6</v>
       </c>
       <c r="EE13" t="n">
         <v>43.4</v>
@@ -32455,7 +32455,7 @@
         <v>-32.9</v>
       </c>
       <c r="IJ13" t="n">
-        <v>4</v>
+        <v>0.8</v>
       </c>
       <c r="IK13" t="n">
         <v>-3.8</v>
@@ -32692,7 +32692,7 @@
         <v>1548.3</v>
       </c>
       <c r="J14" t="n">
-        <v>16.556</v>
+        <v>16</v>
       </c>
       <c r="K14" t="n">
         <v>46.328</v>
@@ -33064,7 +33064,7 @@
         <v>1442.2</v>
       </c>
       <c r="ED14" t="n">
-        <v>13.444</v>
+        <v>14</v>
       </c>
       <c r="EE14" t="n">
         <v>40.3</v>
@@ -33394,7 +33394,7 @@
         <v>106.1</v>
       </c>
       <c r="IJ14" t="n">
-        <v>3.111</v>
+        <v>2</v>
       </c>
       <c r="IK14" t="n">
         <v>2.3</v>
@@ -33631,7 +33631,7 @@
         <v>1459</v>
       </c>
       <c r="J15" t="n">
-        <v>12.111</v>
+        <v>12.2</v>
       </c>
       <c r="K15" t="n">
         <v>48.955</v>
@@ -34003,7 +34003,7 @@
         <v>1487.5</v>
       </c>
       <c r="ED15" t="n">
-        <v>17.889</v>
+        <v>17.8</v>
       </c>
       <c r="EE15" t="n">
         <v>42.2</v>
@@ -34333,7 +34333,7 @@
         <v>-28.5</v>
       </c>
       <c r="IJ15" t="n">
-        <v>-5.778</v>
+        <v>-5.6</v>
       </c>
       <c r="IK15" t="n">
         <v>-0.1</v>
@@ -34570,7 +34570,7 @@
         <v>1368.7</v>
       </c>
       <c r="J16" t="n">
-        <v>2.667</v>
+        <v>2.4</v>
       </c>
       <c r="K16" t="n">
         <v>47.026</v>
@@ -34942,7 +34942,7 @@
         <v>1648.7</v>
       </c>
       <c r="ED16" t="n">
-        <v>27.333</v>
+        <v>27.6</v>
       </c>
       <c r="EE16" t="n">
         <v>45.1</v>
@@ -35272,7 +35272,7 @@
         <v>-280</v>
       </c>
       <c r="IJ16" t="n">
-        <v>-24.667</v>
+        <v>-25.2</v>
       </c>
       <c r="IK16" t="n">
         <v>-7.3</v>
@@ -35509,7 +35509,7 @@
         <v>1534.1</v>
       </c>
       <c r="J17" t="n">
-        <v>14.333</v>
+        <v>14.6</v>
       </c>
       <c r="K17" t="n">
         <v>48.822</v>
@@ -35881,7 +35881,7 @@
         <v>1583.4</v>
       </c>
       <c r="ED17" t="n">
-        <v>15.667</v>
+        <v>15.4</v>
       </c>
       <c r="EE17" t="n">
         <v>41.6</v>
@@ -36211,7 +36211,7 @@
         <v>-49.3</v>
       </c>
       <c r="IJ17" t="n">
-        <v>-1.333</v>
+        <v>-0.8</v>
       </c>
       <c r="IK17" t="n">
         <v>-0.4</v>
@@ -36448,7 +36448,7 @@
         <v>1568.1</v>
       </c>
       <c r="J18" t="n">
-        <v>18.444</v>
+        <v>19.6</v>
       </c>
       <c r="K18" t="n">
         <v>53.087</v>
@@ -36820,7 +36820,7 @@
         <v>1420.9</v>
       </c>
       <c r="ED18" t="n">
-        <v>11.556</v>
+        <v>10.4</v>
       </c>
       <c r="EE18" t="n">
         <v>40.9</v>
@@ -37150,7 +37150,7 @@
         <v>147.2</v>
       </c>
       <c r="IJ18" t="n">
-        <v>6.889</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="IK18" t="n">
         <v>1.8</v>
@@ -37387,7 +37387,7 @@
         <v>1346.9</v>
       </c>
       <c r="J19" t="n">
-        <v>5.667</v>
+        <v>5.1</v>
       </c>
       <c r="K19" t="n">
         <v>45.228</v>
@@ -37759,7 +37759,7 @@
         <v>1587.8</v>
       </c>
       <c r="ED19" t="n">
-        <v>24.333</v>
+        <v>24.9</v>
       </c>
       <c r="EE19" t="n">
         <v>43.2</v>
@@ -38089,7 +38089,7 @@
         <v>-240.9</v>
       </c>
       <c r="IJ19" t="n">
-        <v>-18.667</v>
+        <v>-19.8</v>
       </c>
       <c r="IK19" t="n">
         <v>-3</v>
@@ -38326,7 +38326,7 @@
         <v>1572.6</v>
       </c>
       <c r="J20" t="n">
-        <v>24.889</v>
+        <v>22.5</v>
       </c>
       <c r="K20" t="n">
         <v>52.667</v>
@@ -38698,7 +38698,7 @@
         <v>1529.5</v>
       </c>
       <c r="ED20" t="n">
-        <v>5.111</v>
+        <v>7.5</v>
       </c>
       <c r="EE20" t="n">
         <v>40.1</v>
@@ -39028,7 +39028,7 @@
         <v>43.1</v>
       </c>
       <c r="IJ20" t="n">
-        <v>19.778</v>
+        <v>15</v>
       </c>
       <c r="IK20" t="n">
         <v>2.9</v>
@@ -40836,7 +40836,7 @@
         <v>1532.2</v>
       </c>
       <c r="J2" t="n">
-        <v>9.75</v>
+        <v>12.4</v>
       </c>
       <c r="K2" t="n">
         <v>46.594</v>
@@ -41208,7 +41208,7 @@
         <v>1547.6</v>
       </c>
       <c r="ED2" t="n">
-        <v>20.25</v>
+        <v>17.6</v>
       </c>
       <c r="EE2" t="n">
         <v>40</v>
@@ -41538,7 +41538,7 @@
         <v>-15.4</v>
       </c>
       <c r="IJ2" t="n">
-        <v>-10.5</v>
+        <v>-5.2</v>
       </c>
       <c r="IK2" t="n">
         <v>0.2</v>
@@ -42710,7 +42710,7 @@
         <v>1620</v>
       </c>
       <c r="J4" t="n">
-        <v>16.75</v>
+        <v>17.2</v>
       </c>
       <c r="K4" t="n">
         <v>52.427</v>
@@ -43082,7 +43082,7 @@
         <v>1451.2</v>
       </c>
       <c r="ED4" t="n">
-        <v>13.25</v>
+        <v>12.8</v>
       </c>
       <c r="EE4" t="n">
         <v>39.2</v>
@@ -43412,7 +43412,7 @@
         <v>168.8</v>
       </c>
       <c r="IJ4" t="n">
-        <v>3.5</v>
+        <v>4.4</v>
       </c>
       <c r="IK4" t="n">
         <v>5</v>
@@ -43649,7 +43649,7 @@
         <v>1472.8</v>
       </c>
       <c r="J5" t="n">
-        <v>8</v>
+        <v>7.8</v>
       </c>
       <c r="K5" t="n">
         <v>46.252</v>
@@ -44021,7 +44021,7 @@
         <v>1568.4</v>
       </c>
       <c r="ED5" t="n">
-        <v>22</v>
+        <v>22.2</v>
       </c>
       <c r="EE5" t="n">
         <v>41.6</v>
@@ -44351,7 +44351,7 @@
         <v>-95.59999999999999</v>
       </c>
       <c r="IJ5" t="n">
-        <v>-14</v>
+        <v>-14.4</v>
       </c>
       <c r="IK5" t="n">
         <v>-1.6</v>
@@ -44588,7 +44588,7 @@
         <v>1551.2</v>
       </c>
       <c r="J6" t="n">
-        <v>13.25</v>
+        <v>12.6</v>
       </c>
       <c r="K6" t="n">
         <v>48.664</v>
@@ -44960,7 +44960,7 @@
         <v>1637.8</v>
       </c>
       <c r="ED6" t="n">
-        <v>16.75</v>
+        <v>17.4</v>
       </c>
       <c r="EE6" t="n">
         <v>45</v>
@@ -45290,7 +45290,7 @@
         <v>-86.59999999999999</v>
       </c>
       <c r="IJ6" t="n">
-        <v>-3.5</v>
+        <v>-4.8</v>
       </c>
       <c r="IK6" t="n">
         <v>-5.4</v>
@@ -45527,7 +45527,7 @@
         <v>1451.2</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>7.4</v>
       </c>
       <c r="K7" t="n">
         <v>45.487</v>
@@ -45899,7 +45899,7 @@
         <v>1693.2</v>
       </c>
       <c r="ED7" t="n">
-        <v>28</v>
+        <v>22.6</v>
       </c>
       <c r="EE7" t="n">
         <v>45.6</v>
@@ -46229,7 +46229,7 @@
         <v>-242</v>
       </c>
       <c r="IJ7" t="n">
-        <v>-26</v>
+        <v>-15.2</v>
       </c>
       <c r="IK7" t="n">
         <v>-5.4</v>
@@ -46466,7 +46466,7 @@
         <v>1527</v>
       </c>
       <c r="J8" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="K8" t="n">
         <v>49.709</v>
@@ -46838,7 +46838,7 @@
         <v>1478.6</v>
       </c>
       <c r="ED8" t="n">
-        <v>8.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="EE8" t="n">
         <v>39.6</v>
@@ -47168,7 +47168,7 @@
         <v>48.4</v>
       </c>
       <c r="IJ8" t="n">
-        <v>13</v>
+        <v>12.4</v>
       </c>
       <c r="IK8" t="n">
         <v>3.6</v>
@@ -47405,7 +47405,7 @@
         <v>1621.4</v>
       </c>
       <c r="J9" t="n">
-        <v>13</v>
+        <v>16.4</v>
       </c>
       <c r="K9" t="n">
         <v>52.559</v>
@@ -47777,7 +47777,7 @@
         <v>1470.6</v>
       </c>
       <c r="ED9" t="n">
-        <v>17</v>
+        <v>13.6</v>
       </c>
       <c r="EE9" t="n">
         <v>40.2</v>
@@ -48107,7 +48107,7 @@
         <v>150.8</v>
       </c>
       <c r="IJ9" t="n">
-        <v>-4</v>
+        <v>2.8</v>
       </c>
       <c r="IK9" t="n">
         <v>2.2</v>
@@ -48344,7 +48344,7 @@
         <v>1508.8</v>
       </c>
       <c r="J10" t="n">
-        <v>22.25</v>
+        <v>17.8</v>
       </c>
       <c r="K10" t="n">
         <v>53.818</v>
@@ -48716,7 +48716,7 @@
         <v>1520.2</v>
       </c>
       <c r="ED10" t="n">
-        <v>7.75</v>
+        <v>12.2</v>
       </c>
       <c r="EE10" t="n">
         <v>40.4</v>
@@ -49046,7 +49046,7 @@
         <v>-11.4</v>
       </c>
       <c r="IJ10" t="n">
-        <v>14.5</v>
+        <v>5.6</v>
       </c>
       <c r="IK10" t="n">
         <v>1.8</v>
@@ -49283,7 +49283,7 @@
         <v>1618.2</v>
       </c>
       <c r="J11" t="n">
-        <v>11.5</v>
+        <v>15.2</v>
       </c>
       <c r="K11" t="n">
         <v>50.94</v>
@@ -49655,7 +49655,7 @@
         <v>1490.6</v>
       </c>
       <c r="ED11" t="n">
-        <v>18.5</v>
+        <v>14.8</v>
       </c>
       <c r="EE11" t="n">
         <v>40.6</v>
@@ -49985,7 +49985,7 @@
         <v>127.6</v>
       </c>
       <c r="IJ11" t="n">
-        <v>-7</v>
+        <v>0.4</v>
       </c>
       <c r="IK11" t="n">
         <v>2.6</v>
@@ -50222,7 +50222,7 @@
         <v>1696.6</v>
       </c>
       <c r="J12" t="n">
-        <v>20.25</v>
+        <v>22</v>
       </c>
       <c r="K12" t="n">
         <v>53.937</v>
@@ -50594,7 +50594,7 @@
         <v>1430</v>
       </c>
       <c r="ED12" t="n">
-        <v>9.75</v>
+        <v>8</v>
       </c>
       <c r="EE12" t="n">
         <v>37.6</v>
@@ -50924,7 +50924,7 @@
         <v>266.6</v>
       </c>
       <c r="IJ12" t="n">
-        <v>10.5</v>
+        <v>14</v>
       </c>
       <c r="IK12" t="n">
         <v>8.6</v>
@@ -51161,7 +51161,7 @@
         <v>1505.8</v>
       </c>
       <c r="J13" t="n">
-        <v>20.75</v>
+        <v>16.8</v>
       </c>
       <c r="K13" t="n">
         <v>52.381</v>
@@ -51533,7 +51533,7 @@
         <v>1616.8</v>
       </c>
       <c r="ED13" t="n">
-        <v>9.25</v>
+        <v>13.2</v>
       </c>
       <c r="EE13" t="n">
         <v>44.4</v>
@@ -51863,7 +51863,7 @@
         <v>-111</v>
       </c>
       <c r="IJ13" t="n">
-        <v>11.5</v>
+        <v>3.6</v>
       </c>
       <c r="IK13" t="n">
         <v>-5.2</v>
@@ -52100,7 +52100,7 @@
         <v>1559.2</v>
       </c>
       <c r="J14" t="n">
-        <v>23</v>
+        <v>20.6</v>
       </c>
       <c r="K14" t="n">
         <v>47.352</v>
@@ -52472,7 +52472,7 @@
         <v>1409</v>
       </c>
       <c r="ED14" t="n">
-        <v>7</v>
+        <v>9.4</v>
       </c>
       <c r="EE14" t="n">
         <v>40.2</v>
@@ -52802,7 +52802,7 @@
         <v>150.2</v>
       </c>
       <c r="IJ14" t="n">
-        <v>16</v>
+        <v>11.2</v>
       </c>
       <c r="IK14" t="n">
         <v>3.6</v>
@@ -53039,7 +53039,7 @@
         <v>1532</v>
       </c>
       <c r="J15" t="n">
-        <v>16.75</v>
+        <v>16</v>
       </c>
       <c r="K15" t="n">
         <v>53.747</v>
@@ -53411,7 +53411,7 @@
         <v>1445.4</v>
       </c>
       <c r="ED15" t="n">
-        <v>13.25</v>
+        <v>14</v>
       </c>
       <c r="EE15" t="n">
         <v>41.6</v>
@@ -53741,7 +53741,7 @@
         <v>86.59999999999999</v>
       </c>
       <c r="IJ15" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="IK15" t="n">
         <v>2.2</v>
@@ -53978,7 +53978,7 @@
         <v>1359.2</v>
       </c>
       <c r="J16" t="n">
-        <v>2.25</v>
+        <v>1.8</v>
       </c>
       <c r="K16" t="n">
         <v>47.037</v>
@@ -54350,7 +54350,7 @@
         <v>1588.6</v>
       </c>
       <c r="ED16" t="n">
-        <v>27.75</v>
+        <v>28.2</v>
       </c>
       <c r="EE16" t="n">
         <v>45.6</v>
@@ -54680,7 +54680,7 @@
         <v>-229.4</v>
       </c>
       <c r="IJ16" t="n">
-        <v>-25.5</v>
+        <v>-26.4</v>
       </c>
       <c r="IK16" t="n">
         <v>-7.8</v>
@@ -54917,7 +54917,7 @@
         <v>1554.6</v>
       </c>
       <c r="J17" t="n">
-        <v>11.75</v>
+        <v>12.8</v>
       </c>
       <c r="K17" t="n">
         <v>48.829</v>
@@ -55289,7 +55289,7 @@
         <v>1628.8</v>
       </c>
       <c r="ED17" t="n">
-        <v>18.25</v>
+        <v>17.2</v>
       </c>
       <c r="EE17" t="n">
         <v>43</v>
@@ -55619,7 +55619,7 @@
         <v>-74.2</v>
       </c>
       <c r="IJ17" t="n">
-        <v>-6.5</v>
+        <v>-4.4</v>
       </c>
       <c r="IK17" t="n">
         <v>-1.8</v>
@@ -55856,7 +55856,7 @@
         <v>1598.8</v>
       </c>
       <c r="J18" t="n">
-        <v>21.75</v>
+        <v>23.4</v>
       </c>
       <c r="K18" t="n">
         <v>54.101</v>
@@ -56228,7 +56228,7 @@
         <v>1381.6</v>
       </c>
       <c r="ED18" t="n">
-        <v>8.25</v>
+        <v>6.6</v>
       </c>
       <c r="EE18" t="n">
         <v>40.8</v>
@@ -56558,7 +56558,7 @@
         <v>217.2</v>
       </c>
       <c r="IJ18" t="n">
-        <v>13.5</v>
+        <v>16.8</v>
       </c>
       <c r="IK18" t="n">
         <v>2.4</v>
@@ -56795,7 +56795,7 @@
         <v>1347.8</v>
       </c>
       <c r="J19" t="n">
-        <v>10.5</v>
+        <v>8.4</v>
       </c>
       <c r="K19" t="n">
         <v>45.364</v>
@@ -57167,7 +57167,7 @@
         <v>1599.6</v>
       </c>
       <c r="ED19" t="n">
-        <v>19.5</v>
+        <v>21.6</v>
       </c>
       <c r="EE19" t="n">
         <v>43.6</v>
@@ -57497,7 +57497,7 @@
         <v>-251.8</v>
       </c>
       <c r="IJ19" t="n">
-        <v>-9</v>
+        <v>-13.2</v>
       </c>
       <c r="IK19" t="n">
         <v>-3</v>
@@ -57734,7 +57734,7 @@
         <v>1548.2</v>
       </c>
       <c r="J20" t="n">
-        <v>25</v>
+        <v>20.2</v>
       </c>
       <c r="K20" t="n">
         <v>50.801</v>
@@ -58106,7 +58106,7 @@
         <v>1647</v>
       </c>
       <c r="ED20" t="n">
-        <v>5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="EE20" t="n">
         <v>42.8</v>
@@ -58436,7 +58436,7 @@
         <v>-98.8</v>
       </c>
       <c r="IJ20" t="n">
-        <v>20</v>
+        <v>10.4</v>
       </c>
       <c r="IK20" t="n">
         <v>-2</v>

</xml_diff>